<commit_message>
Sprint 19: dashboard (API and web), landing page after sign-in, video 06 and catalogue row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo/DMS_VIDEO_CATALOGUE.xlsx
+++ b/docs/demo/DMS_VIDEO_CATALOGUE.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -691,6 +691,48 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>06-dms-dashboard</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>19 (dashboard)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2:55</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>The new dashboard, now the first page after sign-in: the four figures (documents you can see, reviews waiting, shared with you, storage), the 30-day upload chart, documents by classification, recent documents and the review queue, links from figures to the library, an employee seeing smaller numbers than the administrator because only visible documents are counted, and the same information laid out by three designs (dense grid with due-soon and activity, focused column, dark with welcome banner).</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>videos/06-dms-dashboard.mp4 .srt .vtt .csv</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting your approval</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint C1: Coolify readiness (web container and proxy, one-address stack, optional virus scan, first-organization command, shipped designs), video 07
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo/DMS_VIDEO_CATALOGUE.xlsx
+++ b/docs/demo/DMS_VIDEO_CATALOGUE.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -733,6 +733,48 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>07-dms-deployment</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>C1 (Coolify readiness)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2:58</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>The stack Coolify will run, shown through its one public address on a local copy: web, service and database behind one address, the two health addresses, creating the first organization and administrator with a single command and a one-time link, the five standard designs already published, creating a category and uploading a first document (virus scan off for the first release), inviting a colleague before email is ready (link command, then four email settings), and what is left for the owner: server, domain, verified email, production bucket. Not deployed to a real server.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>videos/07-dms-deployment.mp4 .srt .vtt .csv</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting your approval</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint M1: DMS on a phone, phase 1 (phone shell, dashboard, documents, upload with camera, approvals, install icons), settings self-check command, video 08
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo/DMS_VIDEO_CATALOGUE.xlsx
+++ b/docs/demo/DMS_VIDEO_CATALOGUE.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,7 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="I1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -522,6 +523,7 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -564,6 +566,7 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -606,6 +609,7 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -648,6 +652,7 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -690,6 +695,7 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -732,6 +738,7 @@
           <t>Awaiting your approval</t>
         </is>
       </c>
+      <c r="I7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -770,6 +777,54 @@
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting your approval</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>08-dms-on-your-phone</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>M1 (phone</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> phase 1)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>3:16</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>The DMS on a phone-sized screen (portrait video): the phone layout with a bottom bar and a red badge for waiting reviews, the dashboard with two figures per row, document search with folded filters, opening a document with versions as cards and an on-screen preview, uploading a photo of a delivery receipt (the camera is stood in for by a saved photo) with the fields the category asks for, approving a review from the phone in a full-screen review, the More list, and how to put it on the home screen on Android and iPhone.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>videos/08-dms-on-your-phone.mp4 .srt .vtt .csv</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Awaiting your approval</t>
         </is>

</xml_diff>